<commit_message>
Automate TC-PERS-006: cross-customer session isolation
Closes the last remaining gap flagged in the QA review: no data
inconsistency check when switching between two different customers in
the same browser session. Logs in as customer A, notes balance, logs
out, logs in as customer B and deposits, logs out, logs back in as A,
and confirms A's balance is unaffected by B's session in between.

Updated manual-test-cases/09 and both READMEs to reflect 81 automated /
0 candidates (was 80 automated / 1 candidate), and regenerated the CSV
and XLSX exports from the updated markdown source.
</commit_message>
<xml_diff>
--- a/manual-test-cases/XYZ-Bank-Test-Cases.xlsx
+++ b/manual-test-cases/XYZ-Bank-Test-Cases.xlsx
@@ -1474,14 +1474,15 @@
   <si>
     <t xml:space="preserve">1. Log in as Customer A, note balance.
 2. Log out.
-3. Log in as Customer B, note balance.
-4. Log back in as Customer A.</t>
-  </si>
-  <si>
-    <t>Customer A's balance after step 4 matches step 1 (unaffected by Customer B's session in between); no cross-contamination of account data.</t>
-  </si>
-  <si>
-    <t>Candidate — extend tests/11-access-and-persistence.spec.ts with a second customer</t>
+3. Log in as Customer B, deposit a known amount.
+4. Log out.
+5. Log back in as Customer A.</t>
+  </si>
+  <si>
+    <t>Customer A's balance after step 5 matches step 1 (unaffected by Customer B's session in between); no cross-contamination of account data.</t>
+  </si>
+  <si>
+    <t>Automated — tests/11-access-and-persistence.spec.ts ("no data inconsistency when switching between two different customers")</t>
   </si>
   <si>
     <t>TC-PERS-007</t>
@@ -4521,8 +4522,8 @@
       <c r="F80" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="G80" s="2" t="s">
-        <v>100</v>
+      <c r="G80" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="H80" s="5" t="s">
         <v>23</v>

</xml_diff>